<commit_message>
Add NCERT EVS Class 3-5 games, experiments, projects and reading; fix level picker
Each Our Wondrous World chapter now carries a game, experiments,
activities, a project with an outcome, extra reading and links to the
same class's other NCERT books. The onboarding level dropdown no longer
re-renders on click, so levels can be changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JToV3XHh1vEGaLuTjTUjQr
</commit_message>
<xml_diff>
--- a/app/DeepKids_Board_Topics_Collated.xlsx
+++ b/app/DeepKids_Board_Topics_Collated.xlsx
@@ -9,12 +9,14 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All boards" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DeepKids Plus · Science L1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Level map" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NCERT EVS · games &amp; projects" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Level map" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All boards'!$A$1:$K$369</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DeepKids Plus · Science L1'!$A$1:$H$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Level map'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NCERT EVS · games &amp; projects'!$A$1:$O$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Level map'!$A$1:$E$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19178,6 +19180,2520 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Level</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Ch</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Chapter</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>What it covers</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Game</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>How to play</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Experiments</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Activities</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Project steps</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>You end up with</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Extra reading</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Other NCERT books (same class)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>DeepKids Plus topics</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Family and Friends</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Kinds of families, relatives and what we call them, roles and shared work at home, friends, generations then and now.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Rishte ki Rail</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>A train leaves 'Me Station' and only correct relations can board. Take turns reading riddle cards ('Your father's sister's son is your…'). Answer in 10 seconds to add a coach to your train; a wrong answer derails it. Longest train wins. Bonus coach for saying the word in a third language.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Hand-span survey: measure the hand span and height of everyone in the family (and a neighbour family). Chart it: do children's hands grow toward their parents' sizes?</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Then-and-Now interview with a grandparent: games, school, food, toys at age 8.
+Chore wheel: list every job at home, see who does it, rotate jobs for one week and talk about how it felt.</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Family Museum Box</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Over 2 weeks collect 5 objects with family stories (an old photo, a utensil, a letter), label each, add a family tree and a recorded elder interview.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>A shoebox museum the child presents to the family</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Grandma's Bag of Stories, Sudha Murty
+The Family Book, Todd Parr</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Santoor Ch 3: Best Friends
+Veena Ch 7: मित्र को पत्र
+Maths Mela Ch 4: Vacation with My Nani Maa</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>B2 My world: how humans live, and why; C6 My family history</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Going to the Mela</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Village fairs: stalls, crafts, toys and rides, buying and selling, crowds and staying safe.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Mela Market</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>You each run a stall (bangles, chaat, toys) with ₹100 in play coins. Draw customer cards with wishes and budgets; sell, give exact change, restock. Surprise cards: 'Lost at the mela: what do you do?' (answer well to earn a coin). First to ₹150 wins.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Firki lab: make paper pinwheels with 4, 6 and 8 blades. Which spins fastest in front of a fan? Does blade size matter?
+Lattu test: spin a top on floor, steel plate and carpet. Time each spin. What slows it down?</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Draw a map of a mela (real or remembered) with stalls, entry, rides and a 'meeting point if lost'.
+Make a traditional toy: a dugdugi (pellet drum) from a paper cup or a chakri.</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Our Mini Mela</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Plan and run a small mela for family or neighbours: 3 stalls, handmade toys, price list, a money log, and a lost-and-found rule.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>A real event, plus a chart of what sold and what was earned</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>StoryWeaver (Pratham Books): search 'mela' for free picture books</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Maths Mela Ch 14: The Surajkund Fair
+Maths Mela Ch 12: Give and Take</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>B2 My world: how humans live, and why; B6 Forces, vibrations &amp; sound</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Celebrating Festivals</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Festivals across India, why they happen when they do (harvests, seasons, the Moon), foods, lights, sharing and celebrating together.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Festival Calendar Race</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>A circle of 12 months on the floor. Draw festival cards (Pongal, Bihu, Onam, Eid, Diwali, Christmas, Baisakhi, Holi, Durga Puja, Gurpurab, Phooldei…). Place each in its month and say why it falls then: harvest, season or Moon. Correct month 1 point, correct reason 2 points, naming the Moon's phase that night 3 points.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Haldi magic: paint with haldi paste, then dab soap water on it. Why does yellow turn red? (Haldi is a natural indicator.)
+Diya and jar: which burns longer, a diya under a small glass or under a big jar? (Adult lights it.)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Festival food map of India: one dish per festival, pinned on a map.
+Mark the next 3 months' full and new moons and find which festivals land on them.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>A Festival of Our Own</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Design a new family festival for this season: what it celebrates, food, decorations, a song, an invitation. Host it.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>A celebration, an invitation card and photos</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Binny's Diwali, Thrity Umrigar
+Lights for Gita, Rachna Gilmore
+Amma, Tell Me About Diwali!, Bhakti Mathur</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 9: प्रकृति पर्व – फूलदेई
+Maths Mela Ch 7: Raksha Bandhan
+Santoor Ch 11: Chanda Mama Counts the Stars</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>B2 My world: how humans live, and why; B5 Cycles in the sky &amp; weather</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Getting to Know Plants</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Kinds of plants (trees, shrubs, herbs, climbers), parts and their jobs, leaf shapes, seeds, what plants need, how we use plants.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Leaf Detective Bingo</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Bingo cards show leaf shapes, edges and vein patterns (heart, needle, toothed, compound, parallel veins). On a 20-minute walk, mark a square only when you hold a matching leaf. First line shouts 'Patta!'. Final round: 'Which part do we eat?' speed quiz with carrot, potato, spinach, cauliflower, rice.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Coloured-water flower: put a white flower or celery stalk in water with food colour. Check after 6 and 24 hours. How did the colour climb?
+Seeds' needs: sow moong in four cups (water + light, no water, dark, cold fridge). Compare after 5 days.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Leaf-rubbing book: 10 leaves, crayon rubbings, names in two languages.
+Adopt a tree: measure its trunk with string, sketch it, visit monthly.</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Kitchen-Garden Pot</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Sow methi or dhaniya, water and measure daily, harvest at about 4 weeks, and cook something with it.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>A harvest, a growth chart and a dish</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>From Seed to Plant, Gail Gibbons
+The Tiny Seed, Eric Carle
+A Seed Is Sleepy, Dianna Hutts Aston</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 5: आम का पेड़
+Veena Ch 13: पेड़ों की अम्मा 'तिमक्का'
+Santoor Ch 4: Out in the Garden</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>A5 Kinds of living things</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Plants and Animals Live Together</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Homes and habitats, how plants and animals depend on each other: food, shelter, pollination and seed spreading.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Web of Life</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Lay 12 living-thing cards on a table (neem tree, bee, myna, earthworm, cow, grass, frog, snake, child…). Take turns joining two with a string and saying how one depends on the other. Then draw a 'Gone!' card: remove that being and every string tied to it. Who is left standing? Rebuild with a rescue plan.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Seed hitchhikers: wear old socks over shoes and walk through grass, then 'plant' the sock in a tray of soil and water it. What grows?
+Be a bee: dab a cotton bud in one flower and touch another. Look with a magnifier at the pollen.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Minibeast hunt under a flowerpot or stone (put everything back).
+Bird-feeder log: who visits, when, what do they eat?</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Wildlife-Friendly Corner</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Set up a water bowl, a feeder, a flowering plant and a bamboo 'insect hotel' on a balcony or garden; keep a 3-week visitor log.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>A working mini habitat and a visitor chart</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Over and Under the Pond, Kate Messner
+Up in the Garden and Down in the Dirt, Kate Messner
+What Do You Do With a Tail Like This?, Steve Jenkins &amp; Robin Page</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 4: बया हमारी चिड़िया रानी!
+Veena Ch 2: चींटी
+Veena Ch 3: कितने पैर?
+Santoor Ch 2: Badal and Moti</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>A5 Kinds of living things; B4 Other beings' worlds: how a bird sees the world; B9 Human impact on the environment</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Living in Harmony</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Living peacefully with people and nature: sharing, solving quarrels, caring for animals and surroundings.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Harmony Village</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>A cooperative game: you both win or lose together. Each round flip a Trouble card (the pond is dirty, friends are quarrelling, a stray dog is hungry, a tree will be cut). Spend your action tokens on fixes and explain your fix to earn a bonus. Keep the Harmony meter above zero for 10 rounds to win.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Noise map: rate the noise in 6 places (kitchen, road, park, temple, bedroom at night) from 1 to 5, or use a phone sound meter. Where do birds sing most?</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Quarrel-fix role play: act out three common fights and try three ways to solve each.
+Ask neighbours how they share water, parking or a park. Draw what you learn.</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Harmony Pact</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Family and child pick one action for 2 weeks (water bowls for street animals, a peace corner, a sharing shelf) and keep a log.</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>A pact poster and a 2-week log</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>The Curious Garden, Peter Brown
+Wangari's Trees of Peace, Jeanette Winter
+Have You Filled a Bucket Today?, Carol McCloud</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 18: हम अनेक किंतु एक
+Veena Ch 12: अपना-अपना काम
+Santoor Ch 8: Thank God</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>B9 Human impact on the environment; C4 What's common between me and other life?; B2 My world: how humans live, and why</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Water – A Precious Gift</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Where water comes from, how we use it, clean and dirty water, saving water, traditional ways of storing rainwater.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Drop Detective</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Each player starts the day with 50 water-drop tokens. Draw activity cards (brushing with the tap running −6, mug bath −15, shower −40, washing a car with a pipe −60) and choose the wiser way where you can. Leak cards hit everyone. The player with the most drops at bedtime wins.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Bottle filter: layer gravel, sand, charcoal and cotton in a cut bottle and pour muddy water through. Clearer, but is it safe to drink? (No, it still needs boiling.)
+Sun vs shade: equal water in two plates. Which dries first, and where did the water go?</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Home water audit: count mugs and buckets used in one day.
+Find out how a stepwell, lake or tank near you stored water.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Rain Catcher</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Make a rain gauge and a rain-collecting container; record rainfall and use the water for plants.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>A working gauge, a collector and a rainfall chart</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>The Water Princess, Susan Verde
+Water Is Water, Miranda Paul
+A Drop Around the World, Barbara McKinney</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Santoor Ch 6: Paper Boats
+Maths Mela Ch 11: Filling and Lifting</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>B8 Nature's events; A4 Materials around me &amp; their properties</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Food We Eat</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Where food comes from, foods of different regions, cooking, sharing meals, eating well.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Thali Builder</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Food cards carry energy, body-building and protective icons. Race to build a balanced thali from your hand; then a twist card asks for a Kerala, Punjabi or Bengali thali using only local foods. Opponent can challenge a card's region.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Starch test: a drop of iodine (Betadine) on potato, rice, bread and cucumber. Which turn blue-black? (Adult; don't eat after.)
+Sprouting chana: weigh 50 g, soak and sprout for 2 days, weigh again. Why heavier?</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Food-origin trail: pick 5 foods at dinner and trace each back to a farm, a tree or an animal.
+Cook a grandparent's recipe together and write it down.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Our Family Cookbook</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Collect 5 recipes from relatives with where each comes from, photos, and one dish the child cooks.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>A handmade or printed recipe booklet</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Gregory, the Terrible Eater, Mitchell Sharmat
+Eating the Alphabet, Lois Ehlert</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Santoor Ch 7: The Big Laddoo
+Veena Ch 6: बीरबल की खिचड़ी
+Veena Ch 14: किसान की होशियारी
+Maths Mela Ch 10: Fun at Class Party!</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>C11 What is food?</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Staying Healthy and Happy</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Keeping clean, eating, sleeping and playing well, feelings, staying happy.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Germ Busters</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>A race track of daily-life squares. Habit squares (washed hands, played outside, slept on time) push you ahead; Germ squares send you back unless you hold a Shield card, which you earn by acting out a healthy habit. First to Bedtime wins.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Glitter germs: glitter on hands, shake hands, then wash with water only vs soap. What's left?
+Heartbeat: count your pulse for 15 seconds, do 30 jumps, count again.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Feelings charades: act out happy, worried, angry, proud; others guess and share when they felt it.
+A one-week sleep and play diary.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>7-Day Healthy Me Challenge</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Track water, sleep, outdoor play, fruit and one kind act each day.</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>A completed challenge chart and a reflection drawing</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Germs Are Not for Sharing, Elizabeth Verdick
+The Busy Body Book, Lizzy Rockwell
+The Color Monster, Anna Llenas</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 10: रस्साकशी</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>C10 Getting sick, getting hurt &amp; getting well; C7 My body parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>This World of Things</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Objects around us and what they are made of, natural vs human-made materials, properties like hard, soft, waterproof, magnetic.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Material Top Trumps</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Make 20 cards of household objects and score each for hardness, bendiness, waterproofness and floating. Each turn, pick a property from your top card; the higher score wins both cards. Test any disputed score for real before deciding.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Raincoat test: drip water on paper, plastic, cotton, wool and foil. Which keep a tissue underneath dry?
+Magnet hunt: which things in the house does a magnet pick up? Are all metals magnetic?</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>'Made of what?' house hunt: find 5 things each of wood, metal, plastic, glass, cloth and clay.
+Old vs new: compare a clay pot and a plastic bottle for keeping water cool.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Material Museum</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Collect, test and label 20 materials with their properties and uses.</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>A museum display the child guides visitors through</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>The Way Things Work Now, David Macaulay (for parent and child together)</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Santoor Ch 5: Talking Toys
+Veena Ch 11: एक जादुई पिटारा
+Maths Mela Ch 2: Toy Joy</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>A4 Materials around me &amp; their properties; A3 What's common between living and non-living?</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Making Things</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>How things are made by hand and by machine, artisans and their tools, turning old things into new.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Inventor's Workshop</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Draw a challenge card ('A bridge that holds 10 coins using only 2 sheets of paper', 'A boat that carries 5 marbles from foil') and a 10-minute timer. Build, test, and score: did it work, how many coins or marbles, how few materials. Swap roles as judge.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Paper strength: flat paper vs folded zig-zag vs rolled tube. How many coins can each hold as a bridge?
+Clay drying: make two small pots, dry one in sun and one in shade. Which cracks?</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Meet an artisan (potter, carpenter, tailor) or watch one at work; list their tools.
+Make a toy from trash using an Arvind Gupta design.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Design, Build, Improve</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Build a working toy (a balloon car or a spinning top), test it, improve it 3 times and record what changed.</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>A working toy and an improvement log</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Rosie Revere, Engineer, Andrea Beaty
+The Most Magnificent Thing, Ashley Spires
+Iggy Peck, Architect, Andrea Beaty</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Santoor Ch 6: Paper Boats
+Maths Mela Ch 5: Fun with Shapes</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>A4 Materials around me &amp; their properties; B6 Forces, vibrations &amp; sound</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Taking Charge of Waste</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Kinds of waste, sorting at home, composting, reducing, reusing and recycling, where waste goes.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Bin Blitz</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>60 seconds on the clock. Flip picture cards and slap each onto the right bin: wet, dry, hazardous, e-waste. Trick cards (a tetra pack, a battery, a used tea bag) are worth double. Beat your last score.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Bury test: bury a banana peel, a paper, a cotton rag and a plastic bag in a pot of soil. Dig up after 3 weeks.
+Start a compost pot with kitchen peels and dry leaves; check its warmth and smell weekly.</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Weigh one day's home waste and sort it.
+Visit or talk to a kabadiwala: what can they sell, what can't they?</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Zero-Waste Week</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Weigh waste for a normal week, then a week of family changes; compare.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Compost, a before-and-after chart and a family pledge</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>One Plastic Bag, Miranda Paul
+Why Should I Recycle?, Jen Green
+The Adventures of a Plastic Bottle, Alison Inches</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>B10 Waste: reduce &amp; manage</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Living Together</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Families and communities, people who help us, animals that live in groups (ants, bees, elephants), why living together helps.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Herd or Alone?</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>You are animals on a grassland. Each round flip a Danger card (a leopard, a drought, a flood). Choose secretly: stay with the herd (safe from predators, but food is shared) or go alone (all the food, but danger hits hard). Score food and lives. After 8 rounds, talk about why elephants, ants and humans live in groups.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Ant teamwork: put a sugar grain and a biscuit crumb near ants. Time how long until the first ant arrives and how many join to carry the crumb.</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Map the helpers in your community and what each does for you.
+Watch a flock of pigeons or crows for 10 minutes: who leads, who keeps watch?</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Community Helpers Story</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Interview 3 helpers (vegetable seller, guard, postman) and make a photo-story.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>A booklet or short video</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Gajapati Kulapati, Ashok Rajagopalan
+Swimmy, Leo Lionni</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Santoor Ch 1: Together We Can
+Maths Mela Ch 9: Equal Groups</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>B2 My world: how humans live, and why</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Exploring Our Neighbourhood</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Maps, directions and landmarks, places and services in the neighbourhood.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Treasure Map Hunt</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>The parent hides a treasure and draws a map with a key, a north arrow and steps ('10 steps north, turn east at the tulsi pot'). The child finds it, then draws a map for the parent. Next level: maps drawn to scale.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Make a compass: rub a needle on a magnet 30 times one way, float it on a leaf in a bowl of water. Which way does it point? Check against the sunrise.</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Neighbourhood walk: mark shops, parks, water taps, a clinic. Draw symbols for each.
+Traffic survey: count vehicles vs trees on your street for 10 minutes.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>My Neighbourhood Atlas</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>A hand-drawn map with key, scale and north arrow, plus photos and notes on 10 places.</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>A folded atlas</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Me on the Map, Joan Sweeney
+Mapping Penny's World, Loreen Leedy</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Maths Mela Ch 2: Hide and Seek
+Maths Mela Ch 13: The Transport Museum</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>B2 My world: how humans live, and why</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Nature Trail</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>The variety of plants and animals around us, food chains, how living things depend on one another.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Food Chain Dominoes</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Each domino has an eater on one half and something eaten on the other, from Indian ecosystems (grass–deer–tiger, plankton–fish–kingfisher, leaf–caterpillar–myna). Match ends to build the longest chain; a 'Decomposer' tile can join any dead end.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Camouflage hunt: scatter 20 green and 20 red paper 'insects' on grass. A partner 'bird' has 30 seconds to pick as many as possible. Which colour survives? Repeat on red soil.</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Nature-trail bingo walk.
+Sketch 10 living things in a field journal with where you found them.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Biodiversity Count</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Mark a 1 m × 1 m square with string in a park or garden; visit weekly for 4 weeks and record every plant and animal.</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>A mini field guide to your square</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>What Do You Do With a Tail Like This?, Steve Jenkins &amp; Robin Page
+The Book of Indian Birds, Salim Ali (reference)</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Santoor Ch 5: The Old Stag
+Veena Ch 2: Bagiche ka Ghongha
+Veena Ch 3: Neem
+Maths Mela Ch 10: Elephants, Tigers, and Leopards</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>A5 Kinds of living things; B4 Other beings' worlds: how a bird sees the world</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Growing Up with Nature</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>How plants and animals grow and change: life cycles, what they need to grow, caring for living things.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Life Cycle Rummy</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Cards show stages of life cycles (egg–caterpillar–pupa–butterfly, seed–seedling–plant–flower, egg–tadpole–froglet–frog, baby–child–adult–elder). Draw and discard like rummy; lay down a full set in the right order and explain one stage.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Bean in a jar: wedge a soaked rajma bean between wet tissue and the glass. Draw the root and shoot every 2 days.
+Measure your own height, hand and foot and compare with your baby measurements.</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Family photo timeline from baby to now.
+Look for eggs, caterpillars or tadpoles on a nature walk (look, don't take).</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Grow and Track</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Grow a marigold or balsam from seed to flower over about 6 weeks, measuring weekly.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>A flowering plant and a growth chart</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>A Butterfly Is Patient, Dianna Hutts Aston
+The Cherry Tree, Ruskin Bond</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 1: Chidiya ka Geet
+Santoor Ch 10: The Swing</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>A5 Kinds of living things; B9 Human impact on the environment</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Food for Health</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>What different foods do for the body, a balanced diet, how food is kept from spoiling.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Nutrient Ninjas</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Food cards show nutrient icons and a price. Challenge cards ask things like 'A tiffin with protein and iron under ₹50' or 'A breakfast for a cricketer'. Build the best answer from your hand; the opponent scores it with the nutrient key.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Spoil or keep? Lemon slices: one plain, one in salt, one in sugar, one in the fridge. Watch for a week (don't eat).
+Iodine starch test on different breakfast foods (adult).</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Read 5 food labels: what's in packaged snacks?
+Plan a week of tiffins together.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Preserve Lab</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Make a small batch of nimbu achar with an elder and compare it with an unsalted control over 3 weeks.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>A jar of pickle and an observation log</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Good Enough to Eat, Lizzy Rockwell</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 4: Hamara Aahar
+Veena Ch 9: Mithaiyon ka Sammelan
+Maths Mela Ch 8: Weigh it, Pour it</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>C11 What is food?</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Happy and Healthy Living</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Exercise, hygiene and sleep, staying safe, preventing illness, feeling well in body and mind.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Body Defence Tower</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Stack defence cards (skin, mucus, fever, white blood cells, vaccine) to build your tower. Each turn the opponent plays germ attack cards; a germ gets through if your tower lacks the right defence. Last tower standing wins.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Bread and hands: touch slices with unwashed, water-washed and soap-washed hands; seal each in a bag for a week (never open).
+Breathing rate before and after skipping for a minute.</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Learn a 5-pose yoga sequence.
+First-aid role play: a cut, a burn, a nosebleed.</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Family Fitness League</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>A 3-week plan with daily points for movement, sleep and water.</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>A league table and handmade medals</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>The Busy Body Book, Lizzy Rockwell
+Germs Are Not for Sharing, Elizabeth Verdick</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>Santoor Ch 7: Fit Body, Fit Mind, Fit Nation
+Santoor Ch 3: Be Smart, Be Safe
+Santoor Ch 8: The Lagori Champions
+Veena Ch 12: Shatranj mein Maat</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>C10 Getting sick, getting hurt &amp; getting well</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>How Things Work</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>How everyday tools and machines work: levers, wheels, pulleys and ramps, pushes and pulls.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Machine Hunt Showdown</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>5 minutes on the clock. Race through the house finding levers, wheels and axles, pulleys, ramps, wedges and screws (scissors, a tap, a door handle, a knife). Show each find to score; the opponent can challenge whether it really is that machine.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Ruler lever: balance a ruler on a pencil and lift a pile of coins with fewer coins by moving the pencil. Where must the pencil go?
+Ramp race: roll a toy car down a board at three heights and measure how far it travels.</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Take apart an old pen or torch (adult checks it's safe) and name the parts.
+Make a pulley with a cotton reel, string and a small bucket.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Chain-Reaction Machine</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Build a 5-step chain (dominoes, a ramp, a ball, a cup, a bell) that rings a bell at the end.</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>A working machine and a video of it</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>The Way Things Work Now, David Macaulay</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>Santoor Ch 2: The Tinkling Bells
+Maths Mela Ch 12: Ticking Clocks and Turning Calendar</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>B6 Forces, vibrations &amp; sound</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>How Things Are Made</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>How things are made from raw materials: cloth, paper, pottery, food; artisans and factories.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Factory Line</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Shuffled step cards for making things (cotton boll to shirt, sugarcane to jaggery, wood to paper, clay to pot). Race to put a set in order; the opponent checks with the answer card. Fastest correct line wins.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Make paper: soak torn newspaper, blend into pulp (adult), spread on a mesh frame, press and dry.
+Butter in a jar: shake cream in a closed jar for 10 minutes. What separates?</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Visit a bakery, potter or tailor and list the steps you see.
+Check 10 things at home: where were they made?</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>From Raw to Ready</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Make one thing from its raw material (handmade paper cards, or cream to butter to ghee) and record each step.</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>A finished product and a process poster</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Charlie Needs a Cloak, Tomie dePaola</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Santoor Ch 12: Maheshwar (known for its handloom weaving)
+Maths Mela Ch 4: Thousands Around Us</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>A4 Materials around me &amp; their properties</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Different Lands, Different Lives</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Different landforms (plains, deserts, coasts, mountains) and how they shape people's homes, food, clothes and work.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Landform Survivor</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Draw a land card (Thar desert, Ladakh, Kerala coast, Gangetic plains). Build a home, food, clothing and transport set from your cards that fits that land. The opponent throws an event at you (sandstorm, snowfall, monsoon flood); survive it with the right card to score.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Insulation test: put an ice cube in boxes lined with mud, paper, cloth and thermocol. Which melts last? Which wall would you want in the desert?
+Sand vs water: two cups under a lamp or in the sun. Which heats faster, and which cools faster at night?</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Make clay models of a mountain, plain, desert and coast.
+Taste one dish from each landform region.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Postcards from India</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Research and draw 4 postcards (one per landform) and build a model of one traditional house.</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>A postcard set and a house model</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>A Gift for Amma: Market Day in India, Meera Sriram
+The Blue Umbrella, Ruskin Bond</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>Santoor Ch 11: A Journey to the Magical Mountains
+Veena Ch 6: Jaipur se Patra
+Veena Ch 8: Onam ke Rang</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>B8 Nature's events; B2 My world: how humans live, and why</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Our Sky</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>The Sun, Moon and stars, shadows, day and night, how the sky changes.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Constellation Connect</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Dot cards of constellations (Saptarishi, Kalpurush/Orion, Vrishchik/Scorpius). Race to join the dots and name it, then read its story card (the seven rishis, Dhruv). Bonus point if you find it in tonight's sky.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Shadow stick: mark a stick's shadow every hour from 9 to 4. When is it shortest?
+Torch and ball: show day and night, then the Moon's phases with a lamp and a ball on a pencil.</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Night-sky watch with a printed star map.
+A one-month moon diary.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Sky Journal and Sundial</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Build a sundial and keep a 30-day moon and sky journal.</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>A working sundial and a sky journal</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Moon! Earth's Best Friend, Stacy McAnulty
+Sun! One in a Billion, Stacy McAnulty
+There's No Place Like Space, Tish Rabe</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 5: Aasman Gira
+Veena Ch 13: Hamara Aditya (India's solar mission)</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>B5 Cycles in the sky &amp; weather; B1 Big Bang &amp; the universe</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Water – The Essence of Life</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Water in living things and daily life, what water dissolves, its forms, the water cycle, scarcity and conservation.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Lake of Two Villages</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>You share one lake of 30 water tokens. Each round, both secretly choose to take 2 (careful) or 5 (greedy) tokens for your fields; then a rain card refills 0–6. If the lake ever empties, both villages lose. Most harvest when the season ends, without emptying the lake, wins. Talk about why sharing rules matter.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>What dissolves? Salt, sugar, sand, oil, haldi, chalk in water. Stir, wait, observe.
+Hidden water: weigh a cucumber slice, dry it in the sun for 2 days, weigh again.</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Trace your home's water from its source to your tap.
+Compare how much water different crops need (rice vs millets).</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Water Heroes Model</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Research a traditional system (stepwell, johad, kund, eri) and build a working rain-harvesting model.</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>A model and a 3-minute talk</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>The Water Princess, Susan Verde
+A River, Marc Martin</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>Santoor Ch 3: The Rainbow
+Veena Ch 12: Ganga ki Kahani
+Maths Mela Ch 8: Weight and Capacity</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>B8 Nature's events; C12 Energy beyond food</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Journey of a River</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>A river's journey from its source to the sea: source, tributary, delta, mouth; fast narrow upper course and slow wide lower course; life along rivers.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>River Run</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>A board from glacier to sea. Roll to move; tributary squares speed you up, dam squares make you wait, pollution squares push you back, the delta is the finish. Each square carries a real fact about the Ganga, Brahmaputra, Narmada or Kaveri.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Stream table: a tray of damp sand on a slope; trickle water from a bottle at the top. Watch channels, bends and a delta form. Try steep vs gentle slopes.</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Trace a river on a map from source to mouth and mark the cities on it.
+Collect river stories, such as the legend of the Kaveri.</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>River Model</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Build a sand or clay river with labelled source, tributaries and delta, and a one-page profile of a river near you.</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>A 3D river model</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>Angry River, Ruskin Bond
+A River, Marc Martin</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 12: Ganga ki Kahani
+Maths Mela Ch 14: Maps and Locations</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>B8 Nature's events</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>The Mystery of Food</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>How food changes: cooking, spoiling, fermenting and digesting (align with the book's focus).</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Food Detective</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Mystery cards give clues (smells sour, bubbles appeared, fuzzy spots, turned sweet when chewed). Use the fewest clues to name what happened: fermentation, spoilage, cooking or digestion. Fewer clues used, more points.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Chew plain roti for 2 minutes: when does it turn sweet?
+Idli batter: keep one bowl warm and one in the fridge overnight. Which rises?
+Milk to curd at room temperature vs in the fridge.</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Ask grandparents how food was preserved without a fridge (sun-drying, pickling).
+Watch a fruit go brown after cutting; does lemon juice stop it?</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Fermentation Lab</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Over one week make curd, idli batter and kanji; photograph and log changes daily.</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Foods to eat and a lab notebook</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Bread, Bread, Bread, Ann Morris</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Maths Mela Ch 6: The Dairy Farm
+Maths Mela Ch 9: Coconut Farm</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>C11 What is food?; B3 The world of microorganisms</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Our School – A Happy Place</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>What makes a learning place happy: people, rules, cleanliness, inclusion. For homeschoolers: your own learning community.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Dream School Draft</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Draft feature cards (library, garden, ramps and lifts, sign-language teacher, sports ground, kitchen) within a budget. Each pick must be justified: who does it help? The opponent can veto once.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Light and sound check: measure how bright and how noisy your learning corner is at different times (use a phone light/sound meter or rate 1–5).</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Interview a friend who goes to school: what makes it happy or hard?
+Agree a set of rules for your homeschool group or siblings.</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Learning-Space Makeover</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Redesign the home learning corner and write a charter for your learning group.</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>A rearranged corner and a signed charter</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>Chuskit Goes to School, Sujatha Padmanabhan
+The Day You Begin, Jacqueline Woodson</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 7: Mera Bachpan</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>B2 My world: how humans live, and why</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Our Vibrant Country</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>India's diversity of languages, foods, dances, festivals and crafts, and what unites us.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>India Quartets</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Each state has 4 cards: language, dance, food, monument. Ask your opponent for a card ('Do you have Assam's dance?'). Collect all four of a state to lay down a quartet. Most quartets wins.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Language sounds: record 'hello' and 'thank you' in 10 Indian languages. Which share words?</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Fill a blank India map with states and one fact each.
+Cook one dish from a state you've never visited.</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>State Exchange</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Video-call or write to a child in another state; make a fact book about each other's state.</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>A two-state fact book</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>A Gift for Amma: Market Day in India, Meera Sriram
+Amma, Take Me to… series, Bhakti Mathur</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 11: Hamare ye Kalamandir
+Veena Ch 8: Kaziranga Rashtriya Udyan ki Yatra</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>B2 My world: how humans live, and why</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Some Unique Places</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Unusual landscapes, rare wildlife and traditions in India (e.g. deserts, mangroves, floating lakes, cold deserts).</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Where in India?</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>A travel guessing game: the opponent reads clues one at a time (floating islands of grass; a white salt desert; mangroves with tigers; bridges grown from tree roots). Guess with fewer clues to score more. Then swap.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Salt from the sea: dissolve salt in water in a shallow plate and leave it in the sun. What's left after 3 days? (This is how salt pans work.)
+Floating island: does a grass mat on a sponge float? What keeps Loktak's phumdis afloat?</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Plan a trip to one unique place: route, budget, packing list.
+Find the animals found only in that place.</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Unique-Place Diorama</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>A shoebox diorama of one place plus a one-minute guide video.</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>A diorama and a video</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>StoryWeaver (Pratham Books): search 'Sundarbans' or 'Ladakh'</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 8: Kaziranga Rashtriya Udyan ki Yatra
+Maths Mela Ch 5: Far and Near
+Maths Mela Ch 14: Maps and Locations</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>B8 Nature's events; B4 Other beings' worlds: how a bird sees the world</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Energy – How Things Work</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Forms of energy, where it comes from (food, fuel, sun, electricity), how devices use it, saving energy.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Energy Chains</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Cards show energy steps (Sun, grass, cow, milk, my muscles, bicycle, dynamo, bulb). Build valid chains where each card's energy turns into the next. Longest chain wins; the opponent can challenge any link.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Pizza-box solar oven: foil, black paper and cling film. Can it melt chocolate? Measure with a thermometer if you have one.
+Rubber-band car: wind more turns, travel further?</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Home energy audit: lights and fans left on, the meter reading each day for a week.
+Find 5 ways energy changes form in the kitchen.</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Solar Cooker Challenge</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Build a solar cooker, test it over 3 days, and cook something simple.</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>A working cooker and a temperature log</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>The Boy Who Harnessed the Wind (picture-book edition), William Kamkwamba &amp; Bryan Mealer
+Energy Island, Allan Drummond</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>Maths Mela Ch 12: Racing Seconds</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>C12 Energy beyond food; B6 Forces, vibrations &amp; sound</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Clothes – How Things are Made</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Fibres (cotton, silk, wool, jute, synthetic), spinning, weaving and dyeing, khadi, how clothes are made.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Fibre Detective</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Mystery fabric scraps in envelopes with clue cards (soaks water fast, comes from a caterpillar, shines, keeps sheep warm). Feel, test with a drop of water, and name the fibre.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Water test: drop water on cotton, polyester, wool and silk. Which soaks it up?
+Natural dyes: boil haldi, onion skins or beetroot (adult) and dye white cloth strips.</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Learn the story of the charkha and khadi.
+Check clothing labels at home: what are your clothes made of?</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Dye and Weave</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Dye cloth or yarn with natural dyes and weave a small mat or bookmark on a cardboard loom.</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>A woven piece</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>Charlie Needs a Cloak, Tomie dePaola</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>Maths Mela Ch 11: Grandmother's Quilt
+Santoor Ch 10: Glass Bangles</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>A4 Materials around me &amp; their properties</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Rhythms of Nature</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Cycles in nature: day and night, seasons, flowering and fruiting times, migration, body clocks.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Nature's Clock</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Event cards (the koel calls, mango trees flower, monsoon arrives, Amur falcons pass through Nagaland, owls hunt) go onto a day wheel or a year wheel. Place each correctly and explain why then; most points wins.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Four o'clock flower (gulbas): note when its flowers open each day for a week.
+Your body clock: rate your energy every 2 hours for 3 days. When are you sharpest?</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Visit one tree every week and record leaves, flowers, fruit and visitors.
+Mark shadow length at noon each week.</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Year Wheel</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>A big circular calendar of local nature events, plus 4 weeks of tree and bird observations.</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>A year-wheel poster</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>The Reasons for Seasons, Gail Gibbons
+A Butterfly Is Patient, Dianna Hutts Aston</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 3: Chaand ka Kurta
+Veena Ch 1: Kiran
+Maths Mela Ch 12: Racing Seconds</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>B5 Cycles in the sky &amp; weather; B4 Other beings' worlds: how a bird sees the world</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Earth – Our Shared Home</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Earth as a shared home for all living things, resources, climate, pollution and caring for the planet.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Planet Keepers</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>A cooperative game. Shared Earth-health tokens start at 20. Each round flip a world event (forest fire, new factory, tree-planting drive) and each player picks one action card. Explain your choice to play it. Finish 10 rounds with Earth-health above 10 to win together.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Greenhouse in a jar: two thermometers in the sun, one covered by a glass jar. Compare after 30 minutes.
+Dust catcher: a Vaseline card outside for 2 days; look with a magnifier.</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>A simple family footprint check: travel, electricity, food waste.
+Debate: should we stop using plastic completely?</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Earth Pledge Campaign</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Choose one family change, measure it for 4 weeks, and present results to neighbours or your learning group.</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>A campaign poster and a results chart</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Earth! My First 4.54 Billion Years, Stacy McAnulty
+The Curious Garden, Peter Brown
+Wangari's Trees of Peace, Jeanette Winter</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>Veena Ch 10: Teen Machhliyan
+Maths Mela Ch 15: Data Through Pictures</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>B9 Human impact on the environment; B1 Big Bang &amp; the universe</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O33"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Plan the year from hours: section time estimates, daily hours per subject, curated activities
Class 3 EVS chapters carry hour estimates for reading, lesson,
worksheet, experiments, activities, game and project, with the days
each spans. Parents set hours per day and days per subject in
onboarding or Plan, and the schedule is built from those hours.
Adds activities curated from StoryCorps, Project WET, Project Learning
Tree, Project WILD, Prindle Institute, NASA JPL, KidsGardening,
Exploratorium, Cornell and Arvind Gupta. Game labels are English.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JToV3XHh1vEGaLuTjTUjQr
</commit_message>
<xml_diff>
--- a/app/DeepKids_Board_Topics_Collated.xlsx
+++ b/app/DeepKids_Board_Topics_Collated.xlsx
@@ -19299,7 +19299,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Rishte ki Rail</t>
+          <t>Relation Railway</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -19530,7 +19530,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Bingo cards show leaf shapes, edges and vein patterns (heart, needle, toothed, compound, parallel veins). On a 20-minute walk, mark a square only when you hold a matching leaf. First line shouts 'Patta!'. Final round: 'Which part do we eat?' speed quiz with carrot, potato, spinach, cauliflower, rice.</t>
+          <t>Bingo cards show leaf shapes, edges and vein patterns (heart, needle, toothed, compound, parallel veins). On a 20-minute walk, mark a square only when you hold a matching leaf. First line shouts 'Leaf!'. Final round: 'Which part do we eat?' speed quiz with carrot, potato, spinach, cauliflower, rice.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Chapter packs: exact day-by-day plans, three worksheet tiers, experiments, activities and other voices
- app/content/SPEC.md defines the pack format; validate_pack.py checks it
- Packs drive lesson days, session counts and parent prep in the app
- Chapter page gets Day plan, Worksheets, Experiments and Other voices tabs
- Cambridge Science now uses the real units from the Learner's Books
- NIOS Environmental Studies Level A (Class 3) and Level B (Class 5) lessons
- First pack: NCERT Class 3 Ch 4 Getting to Know Plants

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JToV3XHh1vEGaLuTjTUjQr
</commit_message>
<xml_diff>
--- a/app/DeepKids_Board_Topics_Collated.xlsx
+++ b/app/DeepKids_Board_Topics_Collated.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Level map" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All boards'!$A$1:$K$369</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All boards'!$A$1:$K$341</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DeepKids Plus · Science L1'!$A$1:$H$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NCERT EVS · games &amp; projects'!$A$1:$O$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Level map'!$A$1:$E$6</definedName>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K369"/>
+  <dimension ref="A1:K341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2186,27 +2186,23 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 1</t>
+          <t>Learner's Book 1 (1st ed., older framework)</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Biology</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>A1 Living &amp; non-living: is the distinction real?; A5 Kinds of living things; B3 The world of microorganisms; B4 Other beings' worlds: how a bird sees the world; C1 Other life inside me; C4 What's common between me and other life?; C7 My body parts; C8 My body's sensors; C11 What is food?</t>
-        </is>
-      </c>
+          <t>Being alive</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2237,27 +2233,23 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 1</t>
+          <t>Learner's Book 1 (1st ed., older framework)</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>Chemistry</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>A3 What's common between living and non-living?; A4 Materials around me &amp; their properties; B10 Waste: reduce &amp; manage</t>
-        </is>
-      </c>
+          <t>Growing plants</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2288,27 +2280,23 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 1</t>
+          <t>Learner's Book 1 (1st ed., older framework)</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Physics</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>B6 Forces, vibrations &amp; sound; B7 Light, colour &amp; shadows; C10 Getting sick, getting hurt &amp; getting well</t>
-        </is>
-      </c>
+          <t>Ourselves</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2339,27 +2327,23 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 1</t>
+          <t>Learner's Book 1 (1st ed., older framework)</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Earth and Space</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>B1 Big Bang &amp; the universe; B5 Cycles in the sky &amp; weather; B8 Nature's events; A4 Materials around me &amp; their properties</t>
-        </is>
-      </c>
+          <t>Materials in my world</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2390,27 +2374,23 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 1</t>
+          <t>Learner's Book 1 (1st ed., older framework)</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Thinking and Working Scientifically</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>A1 Living &amp; non-living: is the distinction real?; A4 Materials around me &amp; their properties; A5 Kinds of living things</t>
-        </is>
-      </c>
+          <t>Pushes and pulls</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr"/>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2441,27 +2421,23 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 1</t>
+          <t>Learner's Book 1 (1st ed., older framework)</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>Science in Context</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>B9 Human impact on the environment; C3 Where humans came from; B2 My world: how humans live, and why</t>
-        </is>
-      </c>
+          <t>Hearing sounds</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2492,23 +2468,23 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 2</t>
+          <t>Learner's Book 2 (2nd ed.)</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Biology</t>
+          <t>Environments and habitats</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2539,23 +2515,23 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 2</t>
+          <t>Learner's Book 2 (2nd ed.)</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Chemistry</t>
+          <t>Forces and movement</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2586,23 +2562,23 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 2</t>
+          <t>Learner's Book 2 (2nd ed.)</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Physics</t>
+          <t>Getting materials right</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2633,23 +2609,23 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 2</t>
+          <t>Learner's Book 2 (2nd ed.)</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Earth and Space</t>
+          <t>Humans and animals grow</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2680,23 +2656,23 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 2</t>
+          <t>Learner's Book 2 (2nd ed.)</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Thinking and Working Scientifically</t>
+          <t>Light</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2727,23 +2703,23 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 2</t>
+          <t>Learner's Book 2 (2nd ed.)</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Science in Context</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2774,23 +2750,23 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 3</t>
+          <t>Learner's Book 3 (1st ed., older framework)</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Biology</t>
+          <t>Looking after plants</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2821,23 +2797,23 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 3</t>
+          <t>Learner's Book 3 (1st ed., older framework)</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Chemistry</t>
+          <t>Looking after ourselves</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2868,23 +2844,23 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 3</t>
+          <t>Learner's Book 3 (1st ed., older framework)</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Physics</t>
+          <t>Living things</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2915,23 +2891,23 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 3</t>
+          <t>Learner's Book 3 (1st ed., older framework)</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>Earth and Space</t>
+          <t>Our five senses</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -2962,23 +2938,23 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 3</t>
+          <t>Learner's Book 3 (1st ed., older framework)</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>Thinking and Working Scientifically</t>
+          <t>Investigating materials</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3009,23 +2985,23 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 3</t>
+          <t>Learner's Book 3 (1st ed., older framework)</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Science in Context</t>
+          <t>Forces and movement</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3056,23 +3032,23 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 4</t>
+          <t>Learner's Book 4 (2nd ed.)</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Biology</t>
+          <t>Living things</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr"/>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3103,23 +3079,23 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 4</t>
+          <t>Learner's Book 4 (2nd ed.)</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Chemistry</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3150,23 +3126,23 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 4</t>
+          <t>Learner's Book 4 (2nd ed.)</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Physics</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr"/>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3197,23 +3173,23 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 4</t>
+          <t>Learner's Book 4 (2nd ed.)</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Earth and Space</t>
+          <t>Earth and its habitats</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr"/>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3244,23 +3220,23 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 4</t>
+          <t>Learner's Book 4 (2nd ed.)</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Thinking and Working Scientifically</t>
+          <t>Light</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr"/>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3291,23 +3267,23 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 4</t>
+          <t>Learner's Book 4 (2nd ed.)</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Science in Context</t>
+          <t>Electricity</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3338,23 +3314,23 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 5</t>
+          <t>Learner's Book 5 (2nd ed.)</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Biology</t>
+          <t>Life cycles of flowering plants</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3385,23 +3361,23 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 5</t>
+          <t>Learner's Book 5 (2nd ed.)</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Chemistry</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3432,23 +3408,23 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 5</t>
+          <t>Learner's Book 5 (2nd ed.)</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Physics</t>
+          <t>States and properties of matter</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr"/>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3479,23 +3455,23 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 5</t>
+          <t>Learner's Book 5 (2nd ed.)</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Earth and Space</t>
+          <t>The digestive system</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr"/>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3526,23 +3502,23 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 5</t>
+          <t>Learner's Book 5 (2nd ed.)</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Thinking and Working Scientifically</t>
+          <t>Forces and magnetism</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr"/>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -3573,23 +3549,23 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Cambridge Primary Science (0097) · Stage 5</t>
+          <t>Learner's Book 5 (2nd ed.)</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Strand</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>Science in Context</t>
+          <t>Seasons and adaptations of plants and animals</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr"/>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>Unit names from Learner's Books to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -13557,7 +13533,7 @@
       </c>
       <c r="K278" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -13608,7 +13584,7 @@
       </c>
       <c r="K279" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -13659,7 +13635,7 @@
       </c>
       <c r="K280" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -13710,7 +13686,7 @@
       </c>
       <c r="K281" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -13761,7 +13737,7 @@
       </c>
       <c r="K282" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -13812,7 +13788,7 @@
       </c>
       <c r="K283" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -13853,7 +13829,7 @@
       </c>
       <c r="I284" s="2" t="inlineStr">
         <is>
-          <t>Water – A Precious Gift</t>
+          <t>Water — A Precious Gift</t>
         </is>
       </c>
       <c r="J284" s="2" t="inlineStr">
@@ -13863,7 +13839,7 @@
       </c>
       <c r="K284" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -13914,7 +13890,7 @@
       </c>
       <c r="K285" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -13965,7 +13941,7 @@
       </c>
       <c r="K286" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14016,7 +13992,7 @@
       </c>
       <c r="K287" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14067,7 +14043,7 @@
       </c>
       <c r="K288" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14118,7 +14094,7 @@
       </c>
       <c r="K289" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14169,7 +14145,7 @@
       </c>
       <c r="K290" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14220,7 +14196,7 @@
       </c>
       <c r="K291" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14271,7 +14247,7 @@
       </c>
       <c r="K292" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14312,7 +14288,7 @@
       </c>
       <c r="I293" s="2" t="inlineStr">
         <is>
-          <t>Growing Up with Nature</t>
+          <t>Growing up with Nature</t>
         </is>
       </c>
       <c r="J293" s="2" t="inlineStr">
@@ -14322,7 +14298,7 @@
       </c>
       <c r="K293" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14373,7 +14349,7 @@
       </c>
       <c r="K294" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14424,7 +14400,7 @@
       </c>
       <c r="K295" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14475,7 +14451,7 @@
       </c>
       <c r="K296" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14516,7 +14492,7 @@
       </c>
       <c r="I297" s="2" t="inlineStr">
         <is>
-          <t>How Things Are Made</t>
+          <t>How Things are Made</t>
         </is>
       </c>
       <c r="J297" s="2" t="inlineStr">
@@ -14526,7 +14502,7 @@
       </c>
       <c r="K297" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14577,7 +14553,7 @@
       </c>
       <c r="K298" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14628,7 +14604,7 @@
       </c>
       <c r="K299" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14669,7 +14645,7 @@
       </c>
       <c r="I300" s="2" t="inlineStr">
         <is>
-          <t>Water – The Essence of Life</t>
+          <t>Water — The Essence of Life</t>
         </is>
       </c>
       <c r="J300" s="2" t="inlineStr">
@@ -14679,7 +14655,7 @@
       </c>
       <c r="K300" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14730,7 +14706,7 @@
       </c>
       <c r="K301" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14781,7 +14757,7 @@
       </c>
       <c r="K302" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14822,7 +14798,7 @@
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>Our School – A Happy Place</t>
+          <t>Our School — A Happy Place</t>
         </is>
       </c>
       <c r="J303" s="2" t="inlineStr">
@@ -14832,7 +14808,7 @@
       </c>
       <c r="K303" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14883,7 +14859,7 @@
       </c>
       <c r="K304" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14934,7 +14910,7 @@
       </c>
       <c r="K305" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -14975,7 +14951,7 @@
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>Energy – How Things Work</t>
+          <t>Energy — How Things Work</t>
         </is>
       </c>
       <c r="J306" s="2" t="inlineStr">
@@ -14985,7 +14961,7 @@
       </c>
       <c r="K306" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15026,7 +15002,7 @@
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>Clothes – How Things are Made</t>
+          <t>Clothes — How Things are Made</t>
         </is>
       </c>
       <c r="J307" s="2" t="inlineStr">
@@ -15036,7 +15012,7 @@
       </c>
       <c r="K307" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15087,7 +15063,7 @@
       </c>
       <c r="K308" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15128,7 +15104,7 @@
       </c>
       <c r="I309" s="2" t="inlineStr">
         <is>
-          <t>Earth – Our Shared Home</t>
+          <t>Earth — Our Shared Home</t>
         </is>
       </c>
       <c r="J309" s="2" t="inlineStr">
@@ -15138,7 +15114,7 @@
       </c>
       <c r="K309" s="2" t="inlineStr">
         <is>
-          <t>Titles from secondary listings</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15154,13 +15130,13 @@
         </is>
       </c>
       <c r="C310" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D310" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E310" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F310" s="2" t="inlineStr">
         <is>
@@ -15169,27 +15145,23 @@
       </c>
       <c r="G310" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies (A 102) · Level A</t>
         </is>
       </c>
       <c r="H310" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>Human existence and the body</t>
-        </is>
-      </c>
-      <c r="J310" s="2" t="inlineStr">
-        <is>
-          <t>C7 My body parts; C3 Where humans came from</t>
-        </is>
-      </c>
+          <t>Concept of Family and Interpersonal Relations</t>
+        </is>
+      </c>
+      <c r="J310" s="2" t="inlineStr"/>
       <c r="K310" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15205,13 +15177,13 @@
         </is>
       </c>
       <c r="C311" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D311" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E311" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F311" s="2" t="inlineStr">
         <is>
@@ -15220,27 +15192,23 @@
       </c>
       <c r="G311" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies (A 102) · Level A</t>
         </is>
       </c>
       <c r="H311" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>Hygiene and health</t>
-        </is>
-      </c>
-      <c r="J311" s="2" t="inlineStr">
-        <is>
-          <t>C10 Getting sick, getting hurt &amp; getting well</t>
-        </is>
-      </c>
+          <t>Our Social Environment</t>
+        </is>
+      </c>
+      <c r="J311" s="2" t="inlineStr"/>
       <c r="K311" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15256,13 +15224,13 @@
         </is>
       </c>
       <c r="C312" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D312" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E312" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F312" s="2" t="inlineStr">
         <is>
@@ -15271,27 +15239,23 @@
       </c>
       <c r="G312" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies (A 102) · Level A</t>
         </is>
       </c>
       <c r="H312" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>Family and kinship</t>
-        </is>
-      </c>
-      <c r="J312" s="2" t="inlineStr">
-        <is>
-          <t>C6 My family history; B2 My world: how humans live, and why</t>
-        </is>
-      </c>
+          <t>Our Festivals</t>
+        </is>
+      </c>
+      <c r="J312" s="2" t="inlineStr"/>
       <c r="K312" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15307,13 +15271,13 @@
         </is>
       </c>
       <c r="C313" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D313" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E313" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F313" s="2" t="inlineStr">
         <is>
@@ -15322,27 +15286,23 @@
       </c>
       <c r="G313" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies (A 102) · Level A</t>
         </is>
       </c>
       <c r="H313" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I313" s="2" t="inlineStr">
         <is>
-          <t>Respect for women and elders</t>
-        </is>
-      </c>
-      <c r="J313" s="2" t="inlineStr">
-        <is>
-          <t>B2 My world: how humans live, and why</t>
-        </is>
-      </c>
+          <t>The Environment</t>
+        </is>
+      </c>
+      <c r="J313" s="2" t="inlineStr"/>
       <c r="K313" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15358,13 +15318,13 @@
         </is>
       </c>
       <c r="C314" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D314" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E314" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F314" s="2" t="inlineStr">
         <is>
@@ -15373,27 +15333,23 @@
       </c>
       <c r="G314" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies (A 102) · Level A</t>
         </is>
       </c>
       <c r="H314" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I314" s="2" t="inlineStr">
         <is>
-          <t>Festivals</t>
-        </is>
-      </c>
-      <c r="J314" s="2" t="inlineStr">
-        <is>
-          <t>B2 My world: how humans live, and why; B5 Cycles in the sky &amp; weather</t>
-        </is>
-      </c>
+          <t>Conservation of Environment</t>
+        </is>
+      </c>
+      <c r="J314" s="2" t="inlineStr"/>
       <c r="K314" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15409,13 +15365,13 @@
         </is>
       </c>
       <c r="C315" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D315" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E315" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F315" s="2" t="inlineStr">
         <is>
@@ -15424,27 +15380,23 @@
       </c>
       <c r="G315" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies (A 102) · Level A</t>
         </is>
       </c>
       <c r="H315" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I315" s="2" t="inlineStr">
         <is>
-          <t>Planets and the sky</t>
-        </is>
-      </c>
-      <c r="J315" s="2" t="inlineStr">
-        <is>
-          <t>B1 Big Bang &amp; the universe; B5 Cycles in the sky &amp; weather</t>
-        </is>
-      </c>
+          <t>Sun-Moon-Stars, Day-Night and Seasons</t>
+        </is>
+      </c>
+      <c r="J315" s="2" t="inlineStr"/>
       <c r="K315" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15460,13 +15412,13 @@
         </is>
       </c>
       <c r="C316" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D316" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E316" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F316" s="2" t="inlineStr">
         <is>
@@ -15475,27 +15427,23 @@
       </c>
       <c r="G316" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies (A 102) · Level A</t>
         </is>
       </c>
       <c r="H316" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>Weather</t>
-        </is>
-      </c>
-      <c r="J316" s="2" t="inlineStr">
-        <is>
-          <t>B5 Cycles in the sky &amp; weather; B8 Nature's events</t>
-        </is>
-      </c>
+          <t>Our Basic Needs</t>
+        </is>
+      </c>
+      <c r="J316" s="2" t="inlineStr"/>
       <c r="K316" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15511,13 +15459,13 @@
         </is>
       </c>
       <c r="C317" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D317" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E317" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F317" s="2" t="inlineStr">
         <is>
@@ -15526,27 +15474,23 @@
       </c>
       <c r="G317" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies (A 102) · Level A</t>
         </is>
       </c>
       <c r="H317" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I317" s="2" t="inlineStr">
         <is>
-          <t>Basic needs and diet</t>
-        </is>
-      </c>
-      <c r="J317" s="2" t="inlineStr">
-        <is>
-          <t>C11 What is food?; C12 Energy beyond food</t>
-        </is>
-      </c>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="J317" s="2" t="inlineStr"/>
       <c r="K317" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15562,13 +15506,13 @@
         </is>
       </c>
       <c r="C318" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D318" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E318" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F318" s="2" t="inlineStr">
         <is>
@@ -15577,27 +15521,23 @@
       </c>
       <c r="G318" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies (A 102) · Level A</t>
         </is>
       </c>
       <c r="H318" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I318" s="2" t="inlineStr">
         <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="J318" s="2" t="inlineStr">
-        <is>
-          <t>B2 My world: how humans live, and why</t>
-        </is>
-      </c>
+          <t>Care and cleanliness of external organs</t>
+        </is>
+      </c>
+      <c r="J318" s="2" t="inlineStr"/>
       <c r="K318" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15613,13 +15553,13 @@
         </is>
       </c>
       <c r="C319" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D319" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E319" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F319" s="2" t="inlineStr">
         <is>
@@ -15628,27 +15568,23 @@
       </c>
       <c r="G319" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies (A 102) · Level A</t>
         </is>
       </c>
       <c r="H319" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I319" s="2" t="inlineStr">
         <is>
-          <t>Communication</t>
-        </is>
-      </c>
-      <c r="J319" s="2" t="inlineStr">
-        <is>
-          <t>B2 My world: how humans live, and why</t>
-        </is>
-      </c>
+          <t>Transport and Communication</t>
+        </is>
+      </c>
+      <c r="J319" s="2" t="inlineStr"/>
       <c r="K319" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15664,13 +15600,13 @@
         </is>
       </c>
       <c r="C320" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D320" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E320" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F320" s="2" t="inlineStr">
         <is>
@@ -15679,27 +15615,23 @@
       </c>
       <c r="G320" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies (A 102) · Level A</t>
         </is>
       </c>
       <c r="H320" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I320" s="2" t="inlineStr">
         <is>
-          <t>Rights: education, information, consumer rights</t>
-        </is>
-      </c>
-      <c r="J320" s="2" t="inlineStr">
-        <is>
-          <t>B2 My world: how humans live, and why</t>
-        </is>
-      </c>
+          <t>National Identity</t>
+        </is>
+      </c>
+      <c r="J320" s="2" t="inlineStr"/>
       <c r="K320" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15715,13 +15647,13 @@
         </is>
       </c>
       <c r="C321" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D321" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E321" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F321" s="2" t="inlineStr">
         <is>
@@ -15730,23 +15662,23 @@
       </c>
       <c r="G321" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies (A 102) · Level A</t>
         </is>
       </c>
       <c r="H321" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I321" s="2" t="inlineStr">
         <is>
-          <t>Human existence and the body</t>
+          <t>Our Social and Economic Environment</t>
         </is>
       </c>
       <c r="J321" s="2" t="inlineStr"/>
       <c r="K321" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15762,38 +15694,38 @@
         </is>
       </c>
       <c r="C322" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D322" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E322" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F322" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G322" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H322" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I322" s="2" t="inlineStr">
         <is>
-          <t>Hygiene and health</t>
+          <t>India's Cultural and Natural Heritage: Its Conservation and Honour</t>
         </is>
       </c>
       <c r="J322" s="2" t="inlineStr"/>
       <c r="K322" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15809,38 +15741,38 @@
         </is>
       </c>
       <c r="C323" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D323" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E323" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F323" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G323" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H323" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I323" s="2" t="inlineStr">
         <is>
-          <t>Family and kinship</t>
+          <t>Peace, Unity and Harmony in Indian Society</t>
         </is>
       </c>
       <c r="J323" s="2" t="inlineStr"/>
       <c r="K323" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15856,38 +15788,38 @@
         </is>
       </c>
       <c r="C324" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D324" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E324" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F324" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G324" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H324" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I324" s="2" t="inlineStr">
         <is>
-          <t>Respect for women and elders</t>
+          <t>Our Social Issues</t>
         </is>
       </c>
       <c r="J324" s="2" t="inlineStr"/>
       <c r="K324" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15903,38 +15835,38 @@
         </is>
       </c>
       <c r="C325" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D325" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E325" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F325" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G325" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H325" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I325" s="2" t="inlineStr">
         <is>
-          <t>Festivals</t>
+          <t>Our Freedom Struggle</t>
         </is>
       </c>
       <c r="J325" s="2" t="inlineStr"/>
       <c r="K325" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15950,38 +15882,38 @@
         </is>
       </c>
       <c r="C326" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D326" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E326" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F326" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G326" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H326" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I326" s="2" t="inlineStr">
         <is>
-          <t>Planets and the sky</t>
+          <t>The States of India and their Physical Features</t>
         </is>
       </c>
       <c r="J326" s="2" t="inlineStr"/>
       <c r="K326" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -15997,38 +15929,38 @@
         </is>
       </c>
       <c r="C327" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D327" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E327" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F327" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G327" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H327" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I327" s="2" t="inlineStr">
         <is>
-          <t>Weather</t>
+          <t>Our Community and Public Administration</t>
         </is>
       </c>
       <c r="J327" s="2" t="inlineStr"/>
       <c r="K327" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -16044,38 +15976,38 @@
         </is>
       </c>
       <c r="C328" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D328" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E328" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F328" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G328" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H328" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>7</t>
         </is>
       </c>
       <c r="I328" s="2" t="inlineStr">
         <is>
-          <t>Basic needs and diet</t>
+          <t>Life of Plants and Animals</t>
         </is>
       </c>
       <c r="J328" s="2" t="inlineStr"/>
       <c r="K328" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -16091,38 +16023,38 @@
         </is>
       </c>
       <c r="C329" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D329" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E329" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F329" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G329" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H329" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I329" s="2" t="inlineStr">
         <is>
-          <t>Transport</t>
+          <t>Soil and Crops</t>
         </is>
       </c>
       <c r="J329" s="2" t="inlineStr"/>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -16138,38 +16070,38 @@
         </is>
       </c>
       <c r="C330" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D330" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E330" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F330" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G330" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H330" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>9</t>
         </is>
       </c>
       <c r="I330" s="2" t="inlineStr">
         <is>
-          <t>Communication</t>
+          <t>Conservation of Soil and Forests</t>
         </is>
       </c>
       <c r="J330" s="2" t="inlineStr"/>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -16185,38 +16117,38 @@
         </is>
       </c>
       <c r="C331" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D331" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E331" s="2" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F331" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G331" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H331" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I331" s="2" t="inlineStr">
         <is>
-          <t>Rights: education, information, consumer rights</t>
+          <t>Sources of Energy and their Importance</t>
         </is>
       </c>
       <c r="J331" s="2" t="inlineStr"/>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -16232,38 +16164,38 @@
         </is>
       </c>
       <c r="C332" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D332" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E332" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F332" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G332" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H332" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>11</t>
         </is>
       </c>
       <c r="I332" s="2" t="inlineStr">
         <is>
-          <t>Human existence and the body</t>
+          <t>Solar System and Earth</t>
         </is>
       </c>
       <c r="J332" s="2" t="inlineStr"/>
       <c r="K332" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -16279,38 +16211,38 @@
         </is>
       </c>
       <c r="C333" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D333" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E333" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F333" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G333" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H333" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>12</t>
         </is>
       </c>
       <c r="I333" s="2" t="inlineStr">
         <is>
-          <t>Hygiene and health</t>
+          <t>Food and Health</t>
         </is>
       </c>
       <c r="J333" s="2" t="inlineStr"/>
       <c r="K333" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -16326,38 +16258,38 @@
         </is>
       </c>
       <c r="C334" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D334" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E334" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F334" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G334" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H334" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>13</t>
         </is>
       </c>
       <c r="I334" s="2" t="inlineStr">
         <is>
-          <t>Family and kinship</t>
+          <t>Internal Organs of the Human Body</t>
         </is>
       </c>
       <c r="J334" s="2" t="inlineStr"/>
       <c r="K334" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -16373,38 +16305,38 @@
         </is>
       </c>
       <c r="C335" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D335" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E335" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F335" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G335" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H335" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>14</t>
         </is>
       </c>
       <c r="I335" s="2" t="inlineStr">
         <is>
-          <t>Respect for women and elders</t>
+          <t>Common Diseases: their Reasons, Prevention and Protection</t>
         </is>
       </c>
       <c r="J335" s="2" t="inlineStr"/>
       <c r="K335" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
@@ -16420,45 +16352,45 @@
         </is>
       </c>
       <c r="C336" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D336" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E336" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F336" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="G336" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
+          <t>Environmental Studies · Level B</t>
         </is>
       </c>
       <c r="H336" s="2" t="inlineStr">
         <is>
-          <t>Theme</t>
+          <t>15</t>
         </is>
       </c>
       <c r="I336" s="2" t="inlineStr">
         <is>
-          <t>Festivals</t>
+          <t>Garbage and Waste Disposal</t>
         </is>
       </c>
       <c r="J336" s="2" t="inlineStr"/>
       <c r="K336" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>From the uploaded book</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>NIOS OBE</t>
+          <t>NCERT / CBSE</t>
         </is>
       </c>
       <c r="B337" s="2" t="inlineStr">
@@ -16467,13 +16399,13 @@
         </is>
       </c>
       <c r="C337" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D337" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E337" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F337" s="2" t="inlineStr">
         <is>
@@ -16482,30 +16414,26 @@
       </c>
       <c r="G337" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H337" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
+          <t>(no book)</t>
+        </is>
+      </c>
+      <c r="H337" s="2" t="inlineStr"/>
       <c r="I337" s="2" t="inlineStr">
         <is>
-          <t>Planets and the sky</t>
-        </is>
-      </c>
-      <c r="J337" s="2" t="inlineStr"/>
-      <c r="K337" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
+          <t>No separate EVS book in Classes 1–2 (NCF 2023): EVS ideas sit inside the language and maths books.</t>
+        </is>
+      </c>
+      <c r="J337" s="2" t="inlineStr">
+        <is>
+          <t>Use DeepKids Science Plus</t>
+        </is>
+      </c>
+      <c r="K337" s="2" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>NIOS OBE</t>
+          <t>NCERT / CBSE</t>
         </is>
       </c>
       <c r="B338" s="2" t="inlineStr">
@@ -16514,13 +16442,13 @@
         </is>
       </c>
       <c r="C338" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D338" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E338" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F338" s="2" t="inlineStr">
         <is>
@@ -16529,25 +16457,21 @@
       </c>
       <c r="G338" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H338" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
+          <t>(no book)</t>
+        </is>
+      </c>
+      <c r="H338" s="2" t="inlineStr"/>
       <c r="I338" s="2" t="inlineStr">
         <is>
-          <t>Weather</t>
-        </is>
-      </c>
-      <c r="J338" s="2" t="inlineStr"/>
-      <c r="K338" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
+          <t>No separate EVS book in Classes 1–2 (NCF 2023): EVS ideas sit inside the language and maths books.</t>
+        </is>
+      </c>
+      <c r="J338" s="2" t="inlineStr">
+        <is>
+          <t>Use DeepKids Science Plus</t>
+        </is>
+      </c>
+      <c r="K338" s="2" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
@@ -16557,42 +16481,44 @@
       </c>
       <c r="B339" s="2" t="inlineStr">
         <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C339" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D339" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E339" s="2" t="n">
-        <v>8</v>
+          <t>Maths</t>
+        </is>
+      </c>
+      <c r="C339" s="2" t="inlineStr">
+        <is>
+          <t>1–5</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>1–5</t>
+        </is>
+      </c>
+      <c r="E339" s="2" t="inlineStr">
+        <is>
+          <t>6–10</t>
+        </is>
       </c>
       <c r="F339" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A / B</t>
         </is>
       </c>
       <c r="G339" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H339" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="H339" s="2" t="inlineStr"/>
       <c r="I339" s="2" t="inlineStr">
         <is>
-          <t>Basic needs and diet</t>
+          <t>Lesson list to be added from NIOS study material</t>
         </is>
       </c>
       <c r="J339" s="2" t="inlineStr"/>
       <c r="K339" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16604,42 +16530,44 @@
       </c>
       <c r="B340" s="2" t="inlineStr">
         <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C340" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D340" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E340" s="2" t="n">
-        <v>8</v>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="C340" s="2" t="inlineStr">
+        <is>
+          <t>1–5</t>
+        </is>
+      </c>
+      <c r="D340" s="2" t="inlineStr">
+        <is>
+          <t>1–5</t>
+        </is>
+      </c>
+      <c r="E340" s="2" t="inlineStr">
+        <is>
+          <t>6–10</t>
+        </is>
       </c>
       <c r="F340" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A / B</t>
         </is>
       </c>
       <c r="G340" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H340" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
+          <t>Language: English</t>
+        </is>
+      </c>
+      <c r="H340" s="2" t="inlineStr"/>
       <c r="I340" s="2" t="inlineStr">
         <is>
-          <t>Transport</t>
+          <t>Lesson list to be added from NIOS study material</t>
         </is>
       </c>
       <c r="J340" s="2" t="inlineStr"/>
       <c r="K340" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -16651,1361 +16579,49 @@
       </c>
       <c r="B341" s="2" t="inlineStr">
         <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C341" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D341" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E341" s="2" t="n">
-        <v>8</v>
+          <t>Hindi</t>
+        </is>
+      </c>
+      <c r="C341" s="2" t="inlineStr">
+        <is>
+          <t>1–5</t>
+        </is>
+      </c>
+      <c r="D341" s="2" t="inlineStr">
+        <is>
+          <t>1–5</t>
+        </is>
+      </c>
+      <c r="E341" s="2" t="inlineStr">
+        <is>
+          <t>6–10</t>
+        </is>
       </c>
       <c r="F341" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A / B</t>
         </is>
       </c>
       <c r="G341" s="2" t="inlineStr">
         <is>
-          <t>Level A · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H341" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
+          <t>Language: Hindi</t>
+        </is>
+      </c>
+      <c r="H341" s="2" t="inlineStr"/>
       <c r="I341" s="2" t="inlineStr">
         <is>
-          <t>Communication</t>
+          <t>Lesson list to be added from NIOS study material</t>
         </is>
       </c>
       <c r="J341" s="2" t="inlineStr"/>
       <c r="K341" s="2" t="inlineStr">
         <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B342" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C342" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D342" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E342" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="F342" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G342" s="2" t="inlineStr">
-        <is>
-          <t>Level A · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H342" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I342" s="2" t="inlineStr">
-        <is>
-          <t>Rights: education, information, consumer rights</t>
-        </is>
-      </c>
-      <c r="J342" s="2" t="inlineStr"/>
-      <c r="K342" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B343" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C343" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D343" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E343" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F343" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G343" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H343" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I343" s="2" t="inlineStr">
-        <is>
-          <t>Human existence and the body</t>
-        </is>
-      </c>
-      <c r="J343" s="2" t="inlineStr"/>
-      <c r="K343" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B344" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C344" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D344" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E344" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F344" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G344" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H344" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I344" s="2" t="inlineStr">
-        <is>
-          <t>Hygiene and health</t>
-        </is>
-      </c>
-      <c r="J344" s="2" t="inlineStr"/>
-      <c r="K344" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="345">
-      <c r="A345" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B345" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C345" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D345" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E345" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F345" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G345" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H345" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I345" s="2" t="inlineStr">
-        <is>
-          <t>Family and kinship</t>
-        </is>
-      </c>
-      <c r="J345" s="2" t="inlineStr"/>
-      <c r="K345" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="346">
-      <c r="A346" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B346" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C346" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D346" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E346" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F346" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G346" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H346" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I346" s="2" t="inlineStr">
-        <is>
-          <t>Respect for women and elders</t>
-        </is>
-      </c>
-      <c r="J346" s="2" t="inlineStr"/>
-      <c r="K346" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B347" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C347" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D347" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E347" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F347" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G347" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H347" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I347" s="2" t="inlineStr">
-        <is>
-          <t>Festivals</t>
-        </is>
-      </c>
-      <c r="J347" s="2" t="inlineStr"/>
-      <c r="K347" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="348">
-      <c r="A348" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B348" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C348" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D348" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E348" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F348" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G348" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H348" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I348" s="2" t="inlineStr">
-        <is>
-          <t>Planets and the sky</t>
-        </is>
-      </c>
-      <c r="J348" s="2" t="inlineStr"/>
-      <c r="K348" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="349">
-      <c r="A349" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B349" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C349" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D349" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E349" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F349" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G349" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H349" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I349" s="2" t="inlineStr">
-        <is>
-          <t>Weather</t>
-        </is>
-      </c>
-      <c r="J349" s="2" t="inlineStr"/>
-      <c r="K349" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="350">
-      <c r="A350" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B350" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C350" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D350" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E350" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F350" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G350" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H350" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I350" s="2" t="inlineStr">
-        <is>
-          <t>Basic needs and diet</t>
-        </is>
-      </c>
-      <c r="J350" s="2" t="inlineStr"/>
-      <c r="K350" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="351">
-      <c r="A351" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B351" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C351" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D351" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E351" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F351" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G351" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H351" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I351" s="2" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="J351" s="2" t="inlineStr"/>
-      <c r="K351" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="352">
-      <c r="A352" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B352" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C352" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D352" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E352" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F352" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G352" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H352" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I352" s="2" t="inlineStr">
-        <is>
-          <t>Communication</t>
-        </is>
-      </c>
-      <c r="J352" s="2" t="inlineStr"/>
-      <c r="K352" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="353">
-      <c r="A353" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B353" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C353" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D353" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E353" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F353" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G353" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H353" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I353" s="2" t="inlineStr">
-        <is>
-          <t>Rights: education, information, consumer rights</t>
-        </is>
-      </c>
-      <c r="J353" s="2" t="inlineStr"/>
-      <c r="K353" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="354">
-      <c r="A354" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B354" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C354" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D354" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E354" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F354" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G354" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H354" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I354" s="2" t="inlineStr">
-        <is>
-          <t>Human existence and the body</t>
-        </is>
-      </c>
-      <c r="J354" s="2" t="inlineStr"/>
-      <c r="K354" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="355">
-      <c r="A355" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B355" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C355" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D355" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E355" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F355" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G355" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H355" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I355" s="2" t="inlineStr">
-        <is>
-          <t>Hygiene and health</t>
-        </is>
-      </c>
-      <c r="J355" s="2" t="inlineStr"/>
-      <c r="K355" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="356">
-      <c r="A356" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B356" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C356" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D356" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E356" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F356" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G356" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H356" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I356" s="2" t="inlineStr">
-        <is>
-          <t>Family and kinship</t>
-        </is>
-      </c>
-      <c r="J356" s="2" t="inlineStr"/>
-      <c r="K356" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="357">
-      <c r="A357" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B357" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C357" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D357" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E357" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F357" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G357" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H357" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I357" s="2" t="inlineStr">
-        <is>
-          <t>Respect for women and elders</t>
-        </is>
-      </c>
-      <c r="J357" s="2" t="inlineStr"/>
-      <c r="K357" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="358">
-      <c r="A358" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B358" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C358" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D358" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E358" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F358" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G358" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H358" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I358" s="2" t="inlineStr">
-        <is>
-          <t>Festivals</t>
-        </is>
-      </c>
-      <c r="J358" s="2" t="inlineStr"/>
-      <c r="K358" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="359">
-      <c r="A359" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B359" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C359" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D359" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E359" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F359" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G359" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H359" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I359" s="2" t="inlineStr">
-        <is>
-          <t>Planets and the sky</t>
-        </is>
-      </c>
-      <c r="J359" s="2" t="inlineStr"/>
-      <c r="K359" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="360">
-      <c r="A360" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B360" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C360" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D360" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E360" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F360" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G360" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H360" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I360" s="2" t="inlineStr">
-        <is>
-          <t>Weather</t>
-        </is>
-      </c>
-      <c r="J360" s="2" t="inlineStr"/>
-      <c r="K360" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="361">
-      <c r="A361" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B361" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C361" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D361" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E361" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F361" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G361" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H361" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I361" s="2" t="inlineStr">
-        <is>
-          <t>Basic needs and diet</t>
-        </is>
-      </c>
-      <c r="J361" s="2" t="inlineStr"/>
-      <c r="K361" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="362">
-      <c r="A362" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B362" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C362" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D362" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E362" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F362" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G362" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H362" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I362" s="2" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="J362" s="2" t="inlineStr"/>
-      <c r="K362" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="363">
-      <c r="A363" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B363" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C363" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D363" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E363" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F363" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G363" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H363" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I363" s="2" t="inlineStr">
-        <is>
-          <t>Communication</t>
-        </is>
-      </c>
-      <c r="J363" s="2" t="inlineStr"/>
-      <c r="K363" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="364">
-      <c r="A364" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B364" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C364" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D364" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E364" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F364" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="G364" s="2" t="inlineStr">
-        <is>
-          <t>Level B · Environmental Study (A-102)</t>
-        </is>
-      </c>
-      <c r="H364" s="2" t="inlineStr">
-        <is>
-          <t>Theme</t>
-        </is>
-      </c>
-      <c r="I364" s="2" t="inlineStr">
-        <is>
-          <t>Rights: education, information, consumer rights</t>
-        </is>
-      </c>
-      <c r="J364" s="2" t="inlineStr"/>
-      <c r="K364" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to add</t>
-        </is>
-      </c>
-    </row>
-    <row r="365">
-      <c r="A365" s="2" t="inlineStr">
-        <is>
-          <t>NCERT / CBSE</t>
-        </is>
-      </c>
-      <c r="B365" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C365" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D365" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E365" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="F365" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G365" s="2" t="inlineStr">
-        <is>
-          <t>(no book)</t>
-        </is>
-      </c>
-      <c r="H365" s="2" t="inlineStr"/>
-      <c r="I365" s="2" t="inlineStr">
-        <is>
-          <t>No separate EVS book in Classes 1–2 (NCF 2023): EVS ideas sit inside the language and maths books.</t>
-        </is>
-      </c>
-      <c r="J365" s="2" t="inlineStr">
-        <is>
-          <t>Use DeepKids Science Plus</t>
-        </is>
-      </c>
-      <c r="K365" s="2" t="inlineStr"/>
-    </row>
-    <row r="366">
-      <c r="A366" s="2" t="inlineStr">
-        <is>
-          <t>NCERT / CBSE</t>
-        </is>
-      </c>
-      <c r="B366" s="2" t="inlineStr">
-        <is>
-          <t>EVS / Science</t>
-        </is>
-      </c>
-      <c r="C366" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D366" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E366" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="F366" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G366" s="2" t="inlineStr">
-        <is>
-          <t>(no book)</t>
-        </is>
-      </c>
-      <c r="H366" s="2" t="inlineStr"/>
-      <c r="I366" s="2" t="inlineStr">
-        <is>
-          <t>No separate EVS book in Classes 1–2 (NCF 2023): EVS ideas sit inside the language and maths books.</t>
-        </is>
-      </c>
-      <c r="J366" s="2" t="inlineStr">
-        <is>
-          <t>Use DeepKids Science Plus</t>
-        </is>
-      </c>
-      <c r="K366" s="2" t="inlineStr"/>
-    </row>
-    <row r="367">
-      <c r="A367" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B367" s="2" t="inlineStr">
-        <is>
-          <t>Maths</t>
-        </is>
-      </c>
-      <c r="C367" s="2" t="inlineStr">
-        <is>
-          <t>1–5</t>
-        </is>
-      </c>
-      <c r="D367" s="2" t="inlineStr">
-        <is>
-          <t>1–5</t>
-        </is>
-      </c>
-      <c r="E367" s="2" t="inlineStr">
-        <is>
-          <t>6–10</t>
-        </is>
-      </c>
-      <c r="F367" s="2" t="inlineStr">
-        <is>
-          <t>A / B</t>
-        </is>
-      </c>
-      <c r="G367" s="2" t="inlineStr">
-        <is>
-          <t>Mathematics</t>
-        </is>
-      </c>
-      <c r="H367" s="2" t="inlineStr"/>
-      <c r="I367" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to be added from NIOS study material</t>
-        </is>
-      </c>
-      <c r="J367" s="2" t="inlineStr"/>
-      <c r="K367" s="2" t="inlineStr">
-        <is>
           <t>Pending</t>
         </is>
       </c>
     </row>
-    <row r="368">
-      <c r="A368" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B368" s="2" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="C368" s="2" t="inlineStr">
-        <is>
-          <t>1–5</t>
-        </is>
-      </c>
-      <c r="D368" s="2" t="inlineStr">
-        <is>
-          <t>1–5</t>
-        </is>
-      </c>
-      <c r="E368" s="2" t="inlineStr">
-        <is>
-          <t>6–10</t>
-        </is>
-      </c>
-      <c r="F368" s="2" t="inlineStr">
-        <is>
-          <t>A / B</t>
-        </is>
-      </c>
-      <c r="G368" s="2" t="inlineStr">
-        <is>
-          <t>Language: English</t>
-        </is>
-      </c>
-      <c r="H368" s="2" t="inlineStr"/>
-      <c r="I368" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to be added from NIOS study material</t>
-        </is>
-      </c>
-      <c r="J368" s="2" t="inlineStr"/>
-      <c r="K368" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="369">
-      <c r="A369" s="2" t="inlineStr">
-        <is>
-          <t>NIOS OBE</t>
-        </is>
-      </c>
-      <c r="B369" s="2" t="inlineStr">
-        <is>
-          <t>Hindi</t>
-        </is>
-      </c>
-      <c r="C369" s="2" t="inlineStr">
-        <is>
-          <t>1–5</t>
-        </is>
-      </c>
-      <c r="D369" s="2" t="inlineStr">
-        <is>
-          <t>1–5</t>
-        </is>
-      </c>
-      <c r="E369" s="2" t="inlineStr">
-        <is>
-          <t>6–10</t>
-        </is>
-      </c>
-      <c r="F369" s="2" t="inlineStr">
-        <is>
-          <t>A / B</t>
-        </is>
-      </c>
-      <c r="G369" s="2" t="inlineStr">
-        <is>
-          <t>Language: Hindi</t>
-        </is>
-      </c>
-      <c r="H369" s="2" t="inlineStr"/>
-      <c r="I369" s="2" t="inlineStr">
-        <is>
-          <t>Lesson list to be added from NIOS study material</t>
-        </is>
-      </c>
-      <c r="J369" s="2" t="inlineStr"/>
-      <c r="K369" s="2" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K369"/>
+  <autoFilter ref="A1:K341"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>